<commit_message>
Reordenamiento de la barra lateral
</commit_message>
<xml_diff>
--- a/ANALISIS DE COMPRAS.xlsx
+++ b/ANALISIS DE COMPRAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RESIDENCIA\MBProject\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF722C6-5B26-49F0-A421-A25F084D2333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8CB012-8496-4F3F-8E00-C03D54CD4A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{792C9C6A-37F1-4EBF-806C-6221D4EB8908}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{792C9C6A-37F1-4EBF-806C-6221D4EB8908}"/>
   </bookViews>
   <sheets>
     <sheet name="COMPRAS - PRESUPUESTO VS EJECUT" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="84">
   <si>
     <t>ID</t>
   </si>
@@ -215,6 +215,72 @@
   </si>
   <si>
     <t>Complejo</t>
+  </si>
+  <si>
+    <t>Enero</t>
+  </si>
+  <si>
+    <t>Factura 123</t>
+  </si>
+  <si>
+    <t>Factura 345</t>
+  </si>
+  <si>
+    <t>Papel</t>
+  </si>
+  <si>
+    <t>Tintas</t>
+  </si>
+  <si>
+    <t>Papel Opalina</t>
+  </si>
+  <si>
+    <t>carpetas</t>
+  </si>
+  <si>
+    <t>Factura 567</t>
+  </si>
+  <si>
+    <t>Factura 789</t>
+  </si>
+  <si>
+    <t>Factura 1011</t>
+  </si>
+  <si>
+    <t>Factura 1233</t>
+  </si>
+  <si>
+    <t>Factura 1455</t>
+  </si>
+  <si>
+    <t>Factura 1677</t>
+  </si>
+  <si>
+    <t>Factura 1899</t>
+  </si>
+  <si>
+    <t>Factura 2121</t>
+  </si>
+  <si>
+    <t>Factura 2343</t>
+  </si>
+  <si>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>Combo box</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Costo</t>
   </si>
 </sst>
 </file>
@@ -274,7 +340,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -414,16 +480,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -433,16 +521,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -757,305 +845,311 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{746CE679-5A99-46E8-9837-7F566FE3CDA4}">
-  <dimension ref="B2:K45"/>
+  <dimension ref="B2:K64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+    </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="16" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="13" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14" t="s">
+      <c r="B4" s="5"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="10" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="14" t="s">
+      <c r="J5" s="10" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B6" s="8"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14" t="s">
+      <c r="B6" s="5"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B7" s="8">
+      <c r="B7" s="5">
         <v>1</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="6">
         <v>100</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B8" s="8">
+      <c r="B8" s="5">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="6">
         <v>2</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="14" t="s">
+      <c r="I8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="8">
+      <c r="B9" s="5">
         <v>3</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="6">
         <v>1500</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="8">
+      <c r="B10" s="5">
         <v>4</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="6">
         <v>50</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B11" s="8">
+      <c r="B11" s="5">
         <v>5</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="6">
         <v>75</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="8">
+      <c r="B12" s="5">
         <v>6</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="6">
         <v>100</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="H12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="14" t="s">
+      <c r="I12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="11">
+      <c r="B13" s="7">
         <v>7</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="9">
         <v>50</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="G13" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J13" s="15" t="s">
+      <c r="J13" s="11" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1374,9 +1468,157 @@
         <v>140</v>
       </c>
     </row>
+    <row r="52" spans="3:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="53" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C53" t="s">
+        <v>62</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H53" s="12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C54" t="s">
+        <v>63</v>
+      </c>
+      <c r="F54" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G54" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H54" s="20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C55" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="56" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C56" t="s">
+        <v>69</v>
+      </c>
+      <c r="F56" t="s">
+        <v>78</v>
+      </c>
+      <c r="G56" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="H56" s="19"/>
+    </row>
+    <row r="57" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C57" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C58" t="s">
+        <v>71</v>
+      </c>
+      <c r="F58" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G58" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="H58" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="I58" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C59" t="s">
+        <v>72</v>
+      </c>
+      <c r="F59" s="18">
+        <v>1</v>
+      </c>
+      <c r="G59" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H59" s="18">
+        <v>1</v>
+      </c>
+      <c r="I59" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C60" t="s">
+        <v>73</v>
+      </c>
+      <c r="F60" s="18">
+        <v>2</v>
+      </c>
+      <c r="G60" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="H60" s="18">
+        <v>2</v>
+      </c>
+      <c r="I60" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="61" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C61" t="s">
+        <v>74</v>
+      </c>
+      <c r="F61" s="18">
+        <v>4</v>
+      </c>
+      <c r="G61" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="H61" s="18">
+        <v>3</v>
+      </c>
+      <c r="I61" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="62" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C62" t="s">
+        <v>75</v>
+      </c>
+      <c r="F62" s="18">
+        <v>56</v>
+      </c>
+      <c r="G62" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="H62" s="18">
+        <v>4</v>
+      </c>
+      <c r="I62" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="63" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C63" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="64" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C64" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="G56:H56"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
cambios de iva y pequeña correccion
</commit_message>
<xml_diff>
--- a/ANALISIS DE COMPRAS.xlsx
+++ b/ANALISIS DE COMPRAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RESIDENCIA\MBProject\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8CB012-8496-4F3F-8E00-C03D54CD4A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67FB238-B4FE-4D38-AF5D-180671DC9CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{792C9C6A-37F1-4EBF-806C-6221D4EB8908}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="85">
   <si>
     <t>ID</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Costo</t>
+  </si>
+  <si>
+    <t>Esto sirve para asignar a que grupo va a pertenecer cada factura ya ejecutad, al asignar un grupo a cada  orden de compra se tendrá un control de que grupo gasta y en auntomatico se va a actualizar los gastos de presupuesto mensual, para conocer en que situación se encuentra el departamento con su presupuesto mensual y/o anual</t>
   </si>
 </sst>
 </file>
@@ -340,7 +343,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -493,11 +496,91 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -512,6 +595,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -527,10 +614,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -845,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{746CE679-5A99-46E8-9837-7F566FE3CDA4}">
-  <dimension ref="B2:K64"/>
+  <dimension ref="B2:K70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
@@ -860,23 +970,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="12" t="s">
         <v>57</v>
       </c>
@@ -946,9 +1056,7 @@
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
-      <c r="J6" s="10" t="s">
-        <v>48</v>
-      </c>
+      <c r="J6" s="10"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="5">
@@ -1487,13 +1595,13 @@
       <c r="C54" t="s">
         <v>63</v>
       </c>
-      <c r="F54" s="20" t="s">
+      <c r="F54" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G54" s="20" t="s">
+      <c r="G54" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H54" s="20" t="s">
+      <c r="H54" s="15" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1509,10 +1617,10 @@
       <c r="F56" t="s">
         <v>78</v>
       </c>
-      <c r="G56" s="19" t="s">
+      <c r="G56" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="H56" s="19"/>
+      <c r="H56" s="20"/>
     </row>
     <row r="57" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C57" t="s">
@@ -1523,16 +1631,16 @@
       <c r="C58" t="s">
         <v>71</v>
       </c>
-      <c r="F58" s="18" t="s">
+      <c r="F58" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="G58" s="18" t="s">
+      <c r="G58" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="H58" s="18" t="s">
+      <c r="H58" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="I58" s="18" t="s">
+      <c r="I58" s="14" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1540,16 +1648,16 @@
       <c r="C59" t="s">
         <v>72</v>
       </c>
-      <c r="F59" s="18">
+      <c r="F59" s="14">
         <v>1</v>
       </c>
-      <c r="G59" s="18" t="s">
+      <c r="G59" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="H59" s="18">
+      <c r="H59" s="14">
         <v>1</v>
       </c>
-      <c r="I59" s="18" t="s">
+      <c r="I59" s="14" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1557,16 +1665,16 @@
       <c r="C60" t="s">
         <v>73</v>
       </c>
-      <c r="F60" s="18">
+      <c r="F60" s="14">
         <v>2</v>
       </c>
-      <c r="G60" s="18" t="s">
+      <c r="G60" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="H60" s="18">
+      <c r="H60" s="14">
         <v>2</v>
       </c>
-      <c r="I60" s="18" t="s">
+      <c r="I60" s="14" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1574,16 +1682,16 @@
       <c r="C61" t="s">
         <v>74</v>
       </c>
-      <c r="F61" s="18">
+      <c r="F61" s="14">
         <v>4</v>
       </c>
-      <c r="G61" s="18" t="s">
+      <c r="G61" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="H61" s="18">
+      <c r="H61" s="14">
         <v>3</v>
       </c>
-      <c r="I61" s="18" t="s">
+      <c r="I61" s="14" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1591,16 +1699,16 @@
       <c r="C62" t="s">
         <v>75</v>
       </c>
-      <c r="F62" s="18">
+      <c r="F62" s="14">
         <v>56</v>
       </c>
-      <c r="G62" s="18" t="s">
+      <c r="G62" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="H62" s="18">
+      <c r="H62" s="14">
         <v>4</v>
       </c>
-      <c r="I62" s="18" t="s">
+      <c r="I62" s="14" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1614,11 +1722,44 @@
         <v>77</v>
       </c>
     </row>
+    <row r="65" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F65" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G65" s="22"/>
+      <c r="H65" s="23"/>
+    </row>
+    <row r="66" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F66" s="24"/>
+      <c r="G66" s="25"/>
+      <c r="H66" s="26"/>
+    </row>
+    <row r="67" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F67" s="24"/>
+      <c r="G67" s="25"/>
+      <c r="H67" s="26"/>
+    </row>
+    <row r="68" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F68" s="24"/>
+      <c r="G68" s="25"/>
+      <c r="H68" s="26"/>
+    </row>
+    <row r="69" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F69" s="24"/>
+      <c r="G69" s="25"/>
+      <c r="H69" s="26"/>
+    </row>
+    <row r="70" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F70" s="27"/>
+      <c r="G70" s="28"/>
+      <c r="H70" s="29"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="G56:H56"/>
+    <mergeCell ref="F65:H70"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>